<commit_message>
Jury mentioned issues resolved
</commit_message>
<xml_diff>
--- a/docs/CourtWala-Project Plan.xlsx
+++ b/docs/CourtWala-Project Plan.xlsx
@@ -86,19 +86,22 @@
     <r>
       <rPr>
         <b/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Segoe UI"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t>user registration/login (Firebase authentication)</t>
     </r>
     <r>
       <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Segoe UI"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -110,19 +113,22 @@
     <r>
       <rPr>
         <b/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Segoe UI"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t>user panel</t>
     </r>
     <r>
       <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Segoe UI"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t xml:space="preserve">: search courts, view details, profile management </t>
     </r>
@@ -137,19 +143,22 @@
     <r>
       <rPr>
         <b/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t>user registration/login (Firebase authentication)</t>
     </r>
     <r>
       <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -161,19 +170,22 @@
     <r>
       <rPr>
         <b/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t>user panel</t>
     </r>
     <r>
       <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="9"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t xml:space="preserve">: search courts, view details, profile management </t>
     </r>
@@ -185,19 +197,22 @@
     <r>
       <rPr>
         <b/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t>user registration/login (Firebase authentication)</t>
     </r>
     <r>
       <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -209,19 +224,22 @@
     <r>
       <rPr>
         <b/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t>user panel</t>
     </r>
     <r>
       <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
         <rFont val="Calibri"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <vertAlign val="baseline"/>
       </rPr>
       <t xml:space="preserve">: search courts, view details, profile management </t>
     </r>
@@ -300,13 +318,124 @@
   </si>
   <si>
     <t>Design and develop UI for player, court owner, and admin panels (Frontend)</t>
+  </si>
+  <si>
+    <t>COURTWALA - 8 MEETING PLAN FYP 1</t>
+  </si>
+  <si>
+    <t>COURTWALA - 8 MEETING PLAN FYP 2</t>
+  </si>
+  <si>
+    <t>Review FYP 1 Internal Evaluation and FYP 2 Project Plan</t>
+  </si>
+  <si>
+    <t>Presented and reviewed the fixes implemented for issues identified by the jury during the FYP-1 evaluation.</t>
+  </si>
+  <si>
+    <t>Presented and reviewed the fixes implemented for issuesidentified by the jury during the FYP-1 evaluation.</t>
+  </si>
+  <si>
+    <t>Fix validation issue all over the app</t>
+  </si>
+  <si>
+    <t>Multiple slot selection fix</t>
+  </si>
+  <si>
+    <t>Fix validation issue all over the app (Jury mentioned issue)</t>
+  </si>
+  <si>
+    <t>Multiple slot selection fix (Jury mentioned issue)</t>
+  </si>
+  <si>
+    <t>Backend Implementation of Advanced Matchmaking Feature</t>
+  </si>
+  <si>
+    <t>Remaining Backend Implementation and UI screens of Matchmaking</t>
+  </si>
+  <si>
+    <t>Backend Implementation of Community Feed</t>
+  </si>
+  <si>
+    <t>Remaining Backend Implementation and UI screens of Community Feed</t>
+  </si>
+  <si>
+    <t>Testing and Final checks, (might add another feature for shop sports items)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final testing, evaluation preparation and Report </t>
+  </si>
+  <si>
+    <t>Hammad and Moiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fix validation issue all over the app </t>
+  </si>
+  <si>
+    <t>Validations fix: Moiz, Slot Selection fix: Marium</t>
+  </si>
+  <si>
+    <t>Backend: Marium, UI screens: Uzair</t>
+  </si>
+  <si>
+    <t>Backend: Marium, UI screens: Hammad</t>
+  </si>
+  <si>
+    <t>Validations fix: Moiz, Slot Selection fix: Hammad</t>
+  </si>
+  <si>
+    <t>Testing and Final checks, (might add an extra feature for shop sports items)</t>
+  </si>
+  <si>
+    <t>Report Update</t>
+  </si>
+  <si>
+    <t>Report: Hammad</t>
+  </si>
+  <si>
+    <t>Marium and Moiz</t>
+  </si>
+  <si>
+    <t>Testing: Marium, Evalutaion: Uzair &amp; Moiz, Report: Hammad</t>
+  </si>
+  <si>
+    <t>Testing: Marium, Evalutaion: Moiz, Report: Hammad</t>
+  </si>
+  <si>
+    <t>Testing: Marium, Evalutaion:  Uzair &amp; Moiz, Report: Hammad</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
+        <rFont val="Arial"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+      </rPr>
+      <t xml:space="preserve">Fix validation issue all over the app </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="false"/>
+        <i val="false"/>
+        <u val="none"/>
+        <rFont val="Calibri"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+      </rPr>
+      <t>, Multiple slot selection fix</t>
+    </r>
+  </si>
+  <si>
+    <t>20% Advance Payment Model Implementation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -407,8 +536,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <color rgb="FFFFE697"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FFFFE697"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri Light"/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri Light"/>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri Light"/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -435,8 +612,18 @@
         <fgColor rgb="FFFFF3CB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE697"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -459,11 +646,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" applyAlignment="1" xfId="0">
       <alignment horizontal="center"/>
@@ -598,6 +800,52 @@
       <alignment vertical="center" horizontal="center"/>
     </xf>
     <xf numFmtId="15" applyNumberFormat="1" fontId="0" applyFont="1" fillId="5" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="15" applyFont="1" fillId="0" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="15" applyFont="1" fillId="0" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="16" applyFont="1" fillId="0" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="17" applyFont="1" fillId="0" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="15" applyFont="1" fillId="6" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="6" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="15" applyFont="1" fillId="7" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="7" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="15" applyFont="1" fillId="5" applyFill="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" applyNumberFormat="1" fontId="2" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" applyNumberFormat="1" fontId="18" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" applyNumberFormat="1" fontId="19" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" applyNumberFormat="1" fontId="19" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" applyNumberFormat="1" fontId="20" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" applyNumberFormat="1" fontId="20" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -922,12 +1170,12 @@
     <col min="3" max="3" width="18.140625" customWidth="1"/>
     <col min="4" max="4" width="18.140625" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="6" max="6" width="59.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" ht="29.25" customFormat="1" s="3">
       <c r="A1" s="40" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -1189,8 +1437,234 @@
         <v>17</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" ht="15.75">
+      <c r="A19" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="41" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" s="41" t="s">
+        <v>4</v>
+      </c>
+      <c r="G19" s="27"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="46">
+        <v>1</v>
+      </c>
+      <c r="B20" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="42">
+        <v>1</v>
+      </c>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44">
+        <v>46081</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="46">
+        <v>2</v>
+      </c>
+      <c r="B21" s="58" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="42">
+        <v>2</v>
+      </c>
+      <c r="D21" s="44">
+        <v>46809</v>
+      </c>
+      <c r="E21" s="44">
+        <v>46095</v>
+      </c>
+      <c r="F21" s="42" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="46"/>
+      <c r="B22" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="42"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="46">
+        <v>3</v>
+      </c>
+      <c r="B23" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="42">
+        <v>3</v>
+      </c>
+      <c r="D23" s="62">
+        <v>46095</v>
+      </c>
+      <c r="E23" s="44">
+        <v>46109</v>
+      </c>
+      <c r="F23" s="43" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="46">
+        <v>4</v>
+      </c>
+      <c r="B24" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="42">
+        <v>4</v>
+      </c>
+      <c r="D24" s="44">
+        <v>46109</v>
+      </c>
+      <c r="E24" s="44">
+        <v>46123</v>
+      </c>
+      <c r="F24" s="42" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="46"/>
+      <c r="B25" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="42"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="43" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="46">
+        <v>5</v>
+      </c>
+      <c r="B26" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="42">
+        <v>5</v>
+      </c>
+      <c r="D26" s="44">
+        <v>46123</v>
+      </c>
+      <c r="E26" s="44">
+        <v>42485</v>
+      </c>
+      <c r="F26" s="43" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="46">
+        <v>6</v>
+      </c>
+      <c r="B27" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="42">
+        <v>6</v>
+      </c>
+      <c r="D27" s="44">
+        <v>46137</v>
+      </c>
+      <c r="E27" s="44">
+        <v>46151</v>
+      </c>
+      <c r="F27" s="43" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="65"/>
+      <c r="B28" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="42"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="43" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="65">
+        <v>7</v>
+      </c>
+      <c r="B29" s="43" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="43">
+        <v>7</v>
+      </c>
+      <c r="D29" s="44">
+        <v>46151</v>
+      </c>
+      <c r="E29" s="49">
+        <v>46165</v>
+      </c>
+      <c r="F29" s="43" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="65">
+        <v>8</v>
+      </c>
+      <c r="B30" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="43">
+        <v>8</v>
+      </c>
+      <c r="D30" s="49">
+        <v>46165</v>
+      </c>
+      <c r="E30" s="49">
+        <v>46179</v>
+      </c>
+      <c r="F30" s="43" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="33">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="C4:C6"/>
@@ -1212,6 +1686,18 @@
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="D13:D14"/>
     <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>